<commit_message>
Add tests for employee and shift management functionality
- Implement tests for employee creation and updates, ensuring proper handling of shifts and login provisioning.
- Add tests for shift saving, validation of break policies, and employee shift assignments.
- Introduce punch correction times logic with corresponding tests to validate check-in and check-out adjustments.
- Create shift form utilities to manage shift configurations, including validation and normalization of shift data.
- Ensure all new features are covered by unit tests to maintain code quality and reliability.
</commit_message>
<xml_diff>
--- a/outputs/payroll-tally-20261007/September-payroll-tally.xlsx
+++ b/outputs/payroll-tally-20261007/September-payroll-tally.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc62266fee4d846b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="2" r:id="Rf87de8b6562b4f80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance issues" sheetId="3" r:id="R9d45965e70374c94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf7f5670bb9374f19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="2" r:id="Rb982fd0a2d9a4f4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance issues" sheetId="3" r:id="Re411ef04373b4d51"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,14 +15,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="200" formatCode="#,##0.00&quot;  &quot;;[Red](#,##0.00)&quot;  &quot;;0.00&quot;  &quot;"/>
     <x:numFmt numFmtId="201" formatCode="0&quot;   &quot;"/>
     <x:numFmt numFmtId="202" formatCode="0.00;[Red](0.00);0.00"/>
     <x:numFmt numFmtId="203" formatCode="dd-mmm-yyyy&quot;  &quot;"/>
     <x:numFmt numFmtId="204" formatCode="0.00"/>
+    <x:numFmt numFmtId="205" formatCode="dd-mmm-yyyy"/>
+    <x:numFmt numFmtId="206" formatCode="h:mm AM/PM"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -61,6 +63,12 @@
       <x:color rgb="FF596B7C"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF253D55"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
   <x:fills count="3">
     <x:fill>
@@ -96,7 +104,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="20">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -153,6 +161,19 @@
     <x:xf numFmtId="204" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -164,7 +185,7 @@
         <x:color rgb="FF805200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2D5"/>
         </x:patternFill>
       </x:fill>
@@ -174,7 +195,7 @@
         <x:color rgb="FF805200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2D5"/>
         </x:patternFill>
       </x:fill>
@@ -184,7 +205,7 @@
         <x:color rgb="FF805200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2D5"/>
         </x:patternFill>
       </x:fill>
@@ -194,7 +215,7 @@
         <x:color rgb="FF805200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2D5"/>
         </x:patternFill>
       </x:fill>
@@ -204,7 +225,7 @@
         <x:color rgb="FF805200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2D5"/>
         </x:patternFill>
       </x:fill>
@@ -516,7 +537,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>HR sheet compared with live Supabase. Read-only snapshot taken 7 Oct 2026, 4:43 pm IST.</x:v>
+        <x:v>HR sheet and confirmed corrections compared with Supabase. Read-only snapshot: 7 Oct 2026, 5:08 pm IST.</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="6"/>
@@ -567,7 +588,7 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
-        <x:v>5 employees could not be matched</x:v>
+        <x:v>5 staff are not yet on the punching machine, as confirmed by the user</x:v>
       </x:c>
       <x:c r="E6" s="2"/>
       <x:c r="F6" s="2"/>
@@ -871,7 +892,7 @@
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="15" t="str">
-        <x:v>Employees not matched</x:v>
+        <x:v>Staff not yet on the punching machine</x:v>
       </x:c>
       <x:c r="B24" s="2"/>
       <x:c r="C24" s="2"/>
@@ -908,7 +929,7 @@
       </x:c>
       <x:c r="C26" s="2"/>
       <x:c r="D26" s="12" t="str">
-        <x:v>Kasinath: HR reports 203 worked hours; Supabase records 184h 45m, with 5 unresolved dates and 1 pending recomputation.</x:v>
+        <x:v>Kasinath: saved 184h 45m; photo replay 185h 37m; HR sheet 203h. The replay still has incomplete punches on 2, 25 and 30 September.</x:v>
       </x:c>
       <x:c r="E26" s="2"/>
       <x:c r="F26" s="2"/>
@@ -940,7 +961,7 @@
       </x:c>
       <x:c r="C28" s="2"/>
       <x:c r="D28" s="12" t="str">
-        <x:v>HR’s biometric notation for 199.45 and 116.55 remains unverified. Both rows are unmatched.</x:v>
+        <x:v>HR confirmed H.MM notation: 199.45 = 199h 45m; 232.4 = 232h 40m. Daily 8h 30m is 8.5 decimal hours.</x:v>
       </x:c>
       <x:c r="E28" s="2"/>
       <x:c r="F28" s="2"/>
@@ -956,7 +977,7 @@
       </x:c>
       <x:c r="C29" s="2"/>
       <x:c r="D29" s="12" t="str">
-        <x:v>The workbook is a comparison of saved records, not a new payroll calculation. No source workbook or live records were changed.</x:v>
+        <x:v>Original HR salary amounts and saved system results remain the reference. The photo is simulated locally; corrections have not been saved to Supabase.</x:v>
       </x:c>
       <x:c r="E29" s="2"/>
       <x:c r="F29" s="2"/>
@@ -1025,7 +1046,7 @@
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
       <x:c r="A35" s="16" t="str">
-        <x:v>System hour totals sum stored minutes before dividing by 60. Differences are System minus HR; original source blanks remain blank.</x:v>
+        <x:v>HR biometric values are H.MM. Convert minutes to decimal hours before comparing with system minutes / 60. Differences are System minus HR.</x:v>
       </x:c>
       <x:c r="B35" s="16"/>
       <x:c r="C35" s="16"/>
@@ -1046,6 +1067,178 @@
       <x:c r="F36" s="16"/>
       <x:c r="G36" s="16"/>
       <x:c r="H36" s="16"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="20" t="str">
+        <x:v>Photo: WhatsApp Image 2026-10-03 at 13.26.31.jpeg. User confirmed Kasinath, September 2026, and 18 September checkout at 12:11 PM.</x:v>
+      </x:c>
+      <x:c r="B37" s="20"/>
+      <x:c r="C37" s="20"/>
+      <x:c r="D37" s="20"/>
+      <x:c r="E37" s="20"/>
+      <x:c r="F37" s="20"/>
+      <x:c r="G37" s="20"/>
+      <x:c r="H37" s="20"/>
+    </x:row>
+    <x:row r="39" ht="30" customHeight="1">
+      <x:c r="A39" s="21" t="str">
+        <x:v>Kasinath’s supplied corrections and local replay</x:v>
+      </x:c>
+      <x:c r="B39" s="2"/>
+      <x:c r="C39" s="2"/>
+      <x:c r="D39" s="2"/>
+    </x:row>
+    <x:row r="40" ht="44" customHeight="1">
+      <x:c r="A40" s="10" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="B40" s="10" t="str">
+        <x:v>Corrected check-in</x:v>
+      </x:c>
+      <x:c r="C40" s="10" t="str">
+        <x:v>Corrected check-out</x:v>
+      </x:c>
+      <x:c r="D40" s="10" t="str">
+        <x:v>Result under the current break rules</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="34" customHeight="1">
+      <x:c r="A41" s="22" t="d">
+        <x:v>2026-09-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B41" s="24" t="n">
+        <x:v>0.3902777777777778</x:v>
+      </x:c>
+      <x:c r="C41" s="24" t="n">
+        <x:v>0.8229166666666666</x:v>
+      </x:c>
+      <x:c r="D41" s="12" t="str">
+        <x:v>8h 56m. Interior punch still missing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="34" customHeight="1">
+      <x:c r="A42" s="22" t="d">
+        <x:v>2026-09-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B42" s="24" t="n">
+        <x:v>0.3861111111111111</x:v>
+      </x:c>
+      <x:c r="C42" s="24" t="n">
+        <x:v>0.7645833333333333</x:v>
+      </x:c>
+      <x:c r="D42" s="12" t="str">
+        <x:v>8h 22m. Punch sequence resolves.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="34" customHeight="1">
+      <x:c r="A43" s="22" t="d">
+        <x:v>2026-09-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B43" s="24" t="n">
+        <x:v>0.4027777777777778</x:v>
+      </x:c>
+      <x:c r="C43" s="24" t="n">
+        <x:v>0.5076388888888889</x:v>
+      </x:c>
+      <x:c r="D43" s="12" t="str">
+        <x:v>2h 31m. Punch sequence resolves.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="34" customHeight="1">
+      <x:c r="A44" s="22" t="d">
+        <x:v>2026-09-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B44" s="24" t="n">
+        <x:v>0.41597222222222224</x:v>
+      </x:c>
+      <x:c r="C44" s="24" t="n">
+        <x:v>0.75625</x:v>
+      </x:c>
+      <x:c r="D44" s="12" t="str">
+        <x:v>6h 25m. Interior punch still missing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="30" customHeight="1">
+      <x:c r="A45" s="2"/>
+      <x:c r="B45" s="2"/>
+      <x:c r="C45" s="2"/>
+      <x:c r="D45" s="2"/>
+    </x:row>
+    <x:row r="46" ht="36" customHeight="1">
+      <x:c r="A46" s="10" t="str">
+        <x:v>September worked time</x:v>
+      </x:c>
+      <x:c r="B46" s="10" t="str">
+        <x:v>Saved system</x:v>
+      </x:c>
+      <x:c r="C46" s="10" t="str">
+        <x:v>Local photo replay</x:v>
+      </x:c>
+      <x:c r="D46" s="10" t="str">
+        <x:v>HR sheet</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="30" customHeight="1">
+      <x:c r="A47" s="2" t="str">
+        <x:v>Hours and minutes</x:v>
+      </x:c>
+      <x:c r="B47" s="2" t="str">
+        <x:v>184h 45m</x:v>
+      </x:c>
+      <x:c r="C47" s="2" t="str">
+        <x:v>185h 37m</x:v>
+      </x:c>
+      <x:c r="D47" s="2" t="str">
+        <x:v>203h 00m</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="30" customHeight="1">
+      <x:c r="A48" s="16" t="str">
+        <x:v>Replay preserves recorded breaks and matching endpoint seconds. It is a provisional comparison, not saved attendance or a payroll result.</x:v>
+      </x:c>
+      <x:c r="B48" s="16"/>
+      <x:c r="C48" s="16"/>
+      <x:c r="D48" s="16"/>
+      <x:c r="E48" s="20"/>
+      <x:c r="F48" s="20"/>
+      <x:c r="G48" s="20"/>
+      <x:c r="H48" s="20"/>
+    </x:row>
+    <x:row r="49" ht="30" customHeight="1">
+      <x:c r="A49" s="16" t="str">
+        <x:v>2 and 25 September need missing break / return evidence. 30 September is not covered by the photo and remains unresolved.</x:v>
+      </x:c>
+      <x:c r="B49" s="16"/>
+      <x:c r="C49" s="16"/>
+      <x:c r="D49" s="16"/>
+      <x:c r="E49" s="20"/>
+      <x:c r="F49" s="20"/>
+      <x:c r="G49" s="20"/>
+      <x:c r="H49" s="20"/>
+    </x:row>
+    <x:row r="50" ht="30" customHeight="1">
+      <x:c r="A50" s="16" t="str">
+        <x:v>The five staff without device enrollment need reviewed manual attendance to reconcile September; missing punches must not become assumed absences.</x:v>
+      </x:c>
+      <x:c r="B50" s="16"/>
+      <x:c r="C50" s="16"/>
+      <x:c r="D50" s="16"/>
+      <x:c r="E50" s="20"/>
+      <x:c r="F50" s="20"/>
+      <x:c r="G50" s="20"/>
+      <x:c r="H50" s="20"/>
+    </x:row>
+    <x:row r="51" ht="30" customHeight="1">
+      <x:c r="A51" s="16" t="str">
+        <x:v>Time conversion example: 199.45 H.MM = 199 + 45/60 = 199.75 decimal hours. The source workbook itself has not been changed.</x:v>
+      </x:c>
+      <x:c r="B51" s="16"/>
+      <x:c r="C51" s="16"/>
+      <x:c r="D51" s="16"/>
+      <x:c r="E51" s="20"/>
+      <x:c r="F51" s="20"/>
+      <x:c r="G51" s="20"/>
+      <x:c r="H51" s="20"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1204,7 +1397,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>September 2026. Amounts in INR. Blank system cells mean unavailable / not configured, not zero. Hour differences remain provisional.</x:v>
+        <x:v>September 2026. INR amounts. HR column H uses H.MM; system hours and differences use decimals. Blank system cells are unavailable, not zero.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1323,7 +1516,7 @@
         <x:v>Salary difference (INR)</x:v>
       </x:c>
       <x:c r="H5" s="10" t="str">
-        <x:v>HR biometric hours</x:v>
+        <x:v>HR biometric time (H.MM)</x:v>
       </x:c>
       <x:c r="I5" s="10" t="str">
         <x:v>System worked minutes</x:v>
@@ -1332,7 +1525,7 @@
         <x:v>System decimal hours</x:v>
       </x:c>
       <x:c r="K5" s="10" t="str">
-        <x:v>Hours difference</x:v>
+        <x:v>Hours difference (decimal)</x:v>
       </x:c>
       <x:c r="L5" s="10" t="str">
         <x:v>HR additions (INR)</x:v>
@@ -1468,7 +1661,7 @@
         <x:v>145.77</x:v>
       </x:c>
       <x:c r="K6" s="17" t="n">
-        <x:f>IF(ISNUMBER(J6),ROUND(J6-H6,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I6),ROUND((I6-(INT(H6)*60+ROUND(MOD(H6,1)*100,0)))/60,2),"")</x:f>
         <x:v>-54.23</x:v>
       </x:c>
       <x:c r="L6" s="11" t="n">
@@ -1583,7 +1776,7 @@
         <x:v>185.05</x:v>
       </x:c>
       <x:c r="K7" s="17" t="n">
-        <x:f>IF(ISNUMBER(J7),ROUND(J7-H7,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I7),ROUND((I7-(INT(H7)*60+ROUND(MOD(H7,1)*100,0)))/60,2),"")</x:f>
         <x:v>-5.95</x:v>
       </x:c>
       <x:c r="L7" s="11" t="n">
@@ -1698,7 +1891,7 @@
         <x:v>79.77</x:v>
       </x:c>
       <x:c r="K8" s="17" t="n">
-        <x:f>IF(ISNUMBER(J8),ROUND(J8-H8,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I8),ROUND((I8-(INT(H8)*60+ROUND(MOD(H8,1)*100,0)))/60,2),"")</x:f>
         <x:v>-6.23</x:v>
       </x:c>
       <x:c r="L8" s="11" t="n">
@@ -1813,7 +2006,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K9" s="17" t="n">
-        <x:f>IF(ISNUMBER(J9),ROUND(J9-H9,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I9),ROUND((I9-(INT(H9)*60+ROUND(MOD(H9,1)*100,0)))/60,2),"")</x:f>
         <x:v>-197</x:v>
       </x:c>
       <x:c r="L9" s="11" t="n">
@@ -1897,7 +2090,7 @@
         <x:v>Salary missing; Inputs missing</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="32" customHeight="1">
+    <x:row r="10" ht="40" customHeight="1">
       <x:c r="A10" s="2" t="n">
         <x:v>7</x:v>
       </x:c>
@@ -1923,7 +2116,7 @@
         <x:f>IF(ISNUMBER(I10),ROUND(I10/60,2),"")</x:f>
       </x:c>
       <x:c r="K10" s="17" t="str">
-        <x:f>IF(ISNUMBER(J10),ROUND(J10-H10,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I10),ROUND((I10-(INT(H10)*60+ROUND(MOD(H10,1)*100,0)))/60,2),"")</x:f>
       </x:c>
       <x:c r="L10" s="11" t="n">
         <x:v>5853</x:v>
@@ -1987,7 +2180,7 @@
       <x:c r="AQ10" s="2" t="str"/>
       <x:c r="AR10" s="12" t="str"/>
       <x:c r="AS10" s="12" t="str">
-        <x:v>Employee identity needs review</x:v>
+        <x:v>Not yet on punching machine; manual attendance and employee setup needed</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="32" customHeight="1">
@@ -2021,7 +2214,7 @@
         <x:v>115.55</x:v>
       </x:c>
       <x:c r="K11" s="17" t="n">
-        <x:f>IF(ISNUMBER(J11),ROUND(J11-H11,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I11),ROUND((I11-(INT(H11)*60+ROUND(MOD(H11,1)*100,0)))/60,2),"")</x:f>
         <x:v>-44.45</x:v>
       </x:c>
       <x:c r="L11" s="11" t="n">
@@ -2138,7 +2331,7 @@
         <x:v>154.92</x:v>
       </x:c>
       <x:c r="K12" s="17" t="n">
-        <x:f>IF(ISNUMBER(J12),ROUND(J12-H12,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I12),ROUND((I12-(INT(H12)*60+ROUND(MOD(H12,1)*100,0)))/60,2),"")</x:f>
         <x:v>-15.08</x:v>
       </x:c>
       <x:c r="L12" s="11" t="n">
@@ -2253,7 +2446,7 @@
         <x:v>214.55</x:v>
       </x:c>
       <x:c r="K13" s="17" t="n">
-        <x:f>IF(ISNUMBER(J13),ROUND(J13-H13,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I13),ROUND((I13-(INT(H13)*60+ROUND(MOD(H13,1)*100,0)))/60,2),"")</x:f>
         <x:v>-8.45</x:v>
       </x:c>
       <x:c r="L13" s="11" t="n">
@@ -2368,7 +2561,7 @@
         <x:v>201.57</x:v>
       </x:c>
       <x:c r="K14" s="17" t="n">
-        <x:f>IF(ISNUMBER(J14),ROUND(J14-H14,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I14),ROUND((I14-(INT(H14)*60+ROUND(MOD(H14,1)*100,0)))/60,2),"")</x:f>
         <x:v>10.57</x:v>
       </x:c>
       <x:c r="L14" s="11" t="n">
@@ -2454,7 +2647,7 @@
         <x:v>Salary missing; Inputs missing</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="32" customHeight="1">
+    <x:row r="15" ht="40" customHeight="1">
       <x:c r="A15" s="2" t="n">
         <x:v>12</x:v>
       </x:c>
@@ -2480,7 +2673,7 @@
         <x:f>IF(ISNUMBER(I15),ROUND(I15/60,2),"")</x:f>
       </x:c>
       <x:c r="K15" s="17" t="str">
-        <x:f>IF(ISNUMBER(J15),ROUND(J15-H15,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I15),ROUND((I15-(INT(H15)*60+ROUND(MOD(H15,1)*100,0)))/60,2),"")</x:f>
       </x:c>
       <x:c r="L15" s="11" t="n">
         <x:v>0</x:v>
@@ -2542,10 +2735,10 @@
       <x:c r="AQ15" s="2" t="str"/>
       <x:c r="AR15" s="12" t="str"/>
       <x:c r="AS15" s="12" t="str">
-        <x:v>Employee identity needs review</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="32" customHeight="1">
+        <x:v>Not yet on punching machine; manual attendance and employee setup needed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="40" customHeight="1">
       <x:c r="A16" s="2" t="n">
         <x:v>13</x:v>
       </x:c>
@@ -2571,7 +2764,7 @@
         <x:f>IF(ISNUMBER(I16),ROUND(I16/60,2),"")</x:f>
       </x:c>
       <x:c r="K16" s="17" t="str">
-        <x:f>IF(ISNUMBER(J16),ROUND(J16-H16,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I16),ROUND((I16-(INT(H16)*60+ROUND(MOD(H16,1)*100,0)))/60,2),"")</x:f>
       </x:c>
       <x:c r="L16" s="11" t="n">
         <x:v>0</x:v>
@@ -2633,10 +2826,10 @@
       <x:c r="AQ16" s="2" t="str"/>
       <x:c r="AR16" s="12" t="str"/>
       <x:c r="AS16" s="12" t="str">
-        <x:v>Employee identity needs review</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="32" customHeight="1">
+        <x:v>Not yet on punching machine; manual attendance and employee setup needed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="46" customHeight="1">
       <x:c r="A17" s="2" t="n">
         <x:v>14</x:v>
       </x:c>
@@ -2670,7 +2863,7 @@
         <x:v>184.75</x:v>
       </x:c>
       <x:c r="K17" s="17" t="n">
-        <x:f>IF(ISNUMBER(J17),ROUND(J17-H17,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I17),ROUND((I17-(INT(H17)*60+ROUND(MOD(H17,1)*100,0)))/60,2),"")</x:f>
         <x:v>-18.25</x:v>
       </x:c>
       <x:c r="L17" s="11" t="n">
@@ -2760,7 +2953,7 @@
         <x:v>Linked device code</x:v>
       </x:c>
       <x:c r="AS17" s="12" t="str">
-        <x:v>Recompute pending</x:v>
+        <x:v>Photo corrections received; local replay 185h 37m. Break punches on 2/25 Sep and 30 Sep still need review.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="32" customHeight="1">
@@ -2794,7 +2987,7 @@
         <x:v>213.88</x:v>
       </x:c>
       <x:c r="K18" s="17" t="n">
-        <x:f>IF(ISNUMBER(J18),ROUND(J18-H18,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I18),ROUND((I18-(INT(H18)*60+ROUND(MOD(H18,1)*100,0)))/60,2),"")</x:f>
         <x:v>-22.12</x:v>
       </x:c>
       <x:c r="L18" s="11" t="n">
@@ -2909,7 +3102,7 @@
         <x:v>191.57</x:v>
       </x:c>
       <x:c r="K19" s="17" t="n">
-        <x:f>IF(ISNUMBER(J19),ROUND(J19-H19,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I19),ROUND((I19-(INT(H19)*60+ROUND(MOD(H19,1)*100,0)))/60,2),"")</x:f>
         <x:v>2.57</x:v>
       </x:c>
       <x:c r="L19" s="11" t="n">
@@ -3028,7 +3221,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K20" s="17" t="n">
-        <x:f>IF(ISNUMBER(J20),ROUND(J20-H20,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I20),ROUND((I20-(INT(H20)*60+ROUND(MOD(H20,1)*100,0)))/60,2),"")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="L20" s="11" t="n">
@@ -3110,7 +3303,7 @@
         <x:v>Salary missing; Inputs missing</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="32" customHeight="1">
+    <x:row r="21" ht="40" customHeight="1">
       <x:c r="A21" s="2" t="n">
         <x:v>18</x:v>
       </x:c>
@@ -3136,7 +3329,7 @@
         <x:f>IF(ISNUMBER(I21),ROUND(I21/60,2),"")</x:f>
       </x:c>
       <x:c r="K21" s="17" t="str">
-        <x:f>IF(ISNUMBER(J21),ROUND(J21-H21,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I21),ROUND((I21-(INT(H21)*60+ROUND(MOD(H21,1)*100,0)))/60,2),"")</x:f>
       </x:c>
       <x:c r="L21" s="11" t="n">
         <x:v>0</x:v>
@@ -3198,7 +3391,7 @@
       <x:c r="AQ21" s="2" t="str"/>
       <x:c r="AR21" s="12" t="str"/>
       <x:c r="AS21" s="12" t="str">
-        <x:v>Employee identity needs review</x:v>
+        <x:v>Not yet on punching machine; manual attendance and employee setup needed</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="32" customHeight="1">
@@ -3232,7 +3425,7 @@
         <x:v>206.58</x:v>
       </x:c>
       <x:c r="K22" s="17" t="n">
-        <x:f>IF(ISNUMBER(J22),ROUND(J22-H22,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I22),ROUND((I22-(INT(H22)*60+ROUND(MOD(H22,1)*100,0)))/60,2),"")</x:f>
         <x:v>-27.42</x:v>
       </x:c>
       <x:c r="L22" s="11" t="n">
@@ -3347,7 +3540,7 @@
         <x:v>197.32</x:v>
       </x:c>
       <x:c r="K23" s="17" t="n">
-        <x:f>IF(ISNUMBER(J23),ROUND(J23-H23,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I23),ROUND((I23-(INT(H23)*60+ROUND(MOD(H23,1)*100,0)))/60,2),"")</x:f>
         <x:v>6.32</x:v>
       </x:c>
       <x:c r="L23" s="11" t="n">
@@ -3464,7 +3657,7 @@
         <x:v>158.73</x:v>
       </x:c>
       <x:c r="K24" s="17" t="n">
-        <x:f>IF(ISNUMBER(J24),ROUND(J24-H24,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I24),ROUND((I24-(INT(H24)*60+ROUND(MOD(H24,1)*100,0)))/60,2),"")</x:f>
         <x:v>-31.27</x:v>
       </x:c>
       <x:c r="L24" s="11" t="n">
@@ -3579,7 +3772,7 @@
         <x:v>183.72</x:v>
       </x:c>
       <x:c r="K25" s="17" t="n">
-        <x:f>IF(ISNUMBER(J25),ROUND(J25-H25,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I25),ROUND((I25-(INT(H25)*60+ROUND(MOD(H25,1)*100,0)))/60,2),"")</x:f>
         <x:v>3.72</x:v>
       </x:c>
       <x:c r="L25" s="11" t="n">
@@ -3694,7 +3887,7 @@
         <x:v>200.03</x:v>
       </x:c>
       <x:c r="K26" s="17" t="n">
-        <x:f>IF(ISNUMBER(J26),ROUND(J26-H26,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I26),ROUND((I26-(INT(H26)*60+ROUND(MOD(H26,1)*100,0)))/60,2),"")</x:f>
         <x:v>-10.97</x:v>
       </x:c>
       <x:c r="L26" s="11" t="n">
@@ -3780,7 +3973,7 @@
         <x:v>Salary missing; Inputs missing</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="32" customHeight="1">
+    <x:row r="27" ht="40" customHeight="1">
       <x:c r="A27" s="2" t="n">
         <x:v>24</x:v>
       </x:c>
@@ -3806,7 +3999,7 @@
         <x:f>IF(ISNUMBER(I27),ROUND(I27/60,2),"")</x:f>
       </x:c>
       <x:c r="K27" s="17" t="str">
-        <x:f>IF(ISNUMBER(J27),ROUND(J27-H27,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I27),ROUND((I27-(INT(H27)*60+ROUND(MOD(H27,1)*100,0)))/60,2),"")</x:f>
       </x:c>
       <x:c r="L27" s="11" t="n">
         <x:v>0</x:v>
@@ -3868,7 +4061,7 @@
       <x:c r="AQ27" s="2" t="str"/>
       <x:c r="AR27" s="12" t="str"/>
       <x:c r="AS27" s="12" t="str">
-        <x:v>Employee identity needs review</x:v>
+        <x:v>Not yet on punching machine; manual attendance and employee setup needed</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="32" customHeight="1">
@@ -3902,7 +4095,7 @@
         <x:v>201.83</x:v>
       </x:c>
       <x:c r="K28" s="17" t="n">
-        <x:f>IF(ISNUMBER(J28),ROUND(J28-H28,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I28),ROUND((I28-(INT(H28)*60+ROUND(MOD(H28,1)*100,0)))/60,2),"")</x:f>
         <x:v>-20.17</x:v>
       </x:c>
       <x:c r="L28" s="11" t="n">
@@ -4017,7 +4210,7 @@
         <x:v>190.53</x:v>
       </x:c>
       <x:c r="K29" s="17" t="n">
-        <x:f>IF(ISNUMBER(J29),ROUND(J29-H29,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I29),ROUND((I29-(INT(H29)*60+ROUND(MOD(H29,1)*100,0)))/60,2),"")</x:f>
         <x:v>3.53</x:v>
       </x:c>
       <x:c r="L29" s="11" t="n">
@@ -4136,7 +4329,7 @@
         <x:v>215.18</x:v>
       </x:c>
       <x:c r="K30" s="17" t="n">
-        <x:f>IF(ISNUMBER(J30),ROUND(J30-H30,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I30),ROUND((I30-(INT(H30)*60+ROUND(MOD(H30,1)*100,0)))/60,2),"")</x:f>
         <x:v>-2.82</x:v>
       </x:c>
       <x:c r="L30" s="11" t="n">
@@ -4255,7 +4448,7 @@
         <x:v>226.87</x:v>
       </x:c>
       <x:c r="K31" s="17" t="n">
-        <x:f>IF(ISNUMBER(J31),ROUND(J31-H31,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I31),ROUND((I31-(INT(H31)*60+ROUND(MOD(H31,1)*100,0)))/60,2),"")</x:f>
         <x:v>-5.13</x:v>
       </x:c>
       <x:c r="L31" s="11" t="n">
@@ -4372,7 +4565,7 @@
         <x:v>192.43</x:v>
       </x:c>
       <x:c r="K32" s="17" t="n">
-        <x:f>IF(ISNUMBER(J32),ROUND(J32-H32,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I32),ROUND((I32-(INT(H32)*60+ROUND(MOD(H32,1)*100,0)))/60,2),"")</x:f>
         <x:v>3.43</x:v>
       </x:c>
       <x:c r="L32" s="11" t="n">
@@ -4489,7 +4682,7 @@
         <x:v>214.97</x:v>
       </x:c>
       <x:c r="K33" s="17" t="n">
-        <x:f>IF(ISNUMBER(J33),ROUND(J33-H33,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I33),ROUND((I33-(INT(H33)*60+ROUND(MOD(H33,1)*100,0)))/60,2),"")</x:f>
         <x:v>6.97</x:v>
       </x:c>
       <x:c r="L33" s="11" t="n">
@@ -4606,7 +4799,7 @@
         <x:v>145.75</x:v>
       </x:c>
       <x:c r="K34" s="17" t="n">
-        <x:f>IF(ISNUMBER(J34),ROUND(J34-H34,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I34),ROUND((I34-(INT(H34)*60+ROUND(MOD(H34,1)*100,0)))/60,2),"")</x:f>
         <x:v>-42.25</x:v>
       </x:c>
       <x:c r="L34" s="11" t="n">
@@ -4723,7 +4916,7 @@
         <x:v>194.67</x:v>
       </x:c>
       <x:c r="K35" s="17" t="n">
-        <x:f>IF(ISNUMBER(J35),ROUND(J35-H35,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I35),ROUND((I35-(INT(H35)*60+ROUND(MOD(H35,1)*100,0)))/60,2),"")</x:f>
         <x:v>1.67</x:v>
       </x:c>
       <x:c r="L35" s="11" t="n">
@@ -4840,7 +5033,7 @@
         <x:v>203.33</x:v>
       </x:c>
       <x:c r="K36" s="17" t="n">
-        <x:f>IF(ISNUMBER(J36),ROUND(J36-H36,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I36),ROUND((I36-(INT(H36)*60+ROUND(MOD(H36,1)*100,0)))/60,2),"")</x:f>
         <x:v>-1.67</x:v>
       </x:c>
       <x:c r="L36" s="11" t="n">
@@ -4955,7 +5148,7 @@
         <x:v>168.5</x:v>
       </x:c>
       <x:c r="K37" s="17" t="n">
-        <x:f>IF(ISNUMBER(J37),ROUND(J37-H37,2),"")</x:f>
+        <x:f>IF(ISNUMBER(I37),ROUND((I37-(INT(H37)*60+ROUND(MOD(H37,1)*100,0)))/60,2),"")</x:f>
         <x:v>-36.5</x:v>
       </x:c>
       <x:c r="L37" s="11" t="n">
@@ -5063,7 +5256,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R974af6edd93e402a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R100e0a02e0a24ee0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8104,7 +8297,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5468a73eff614f83"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raec6073497a6469e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>